<commit_message>
updated ETF portfolio optimization
</commit_message>
<xml_diff>
--- a/template_etf_input.xlsx
+++ b/template_etf_input.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28227"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zypub\PycharmProjects\sport\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C910532F-100F-4B6D-A660-F1A1346C346F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" activeTab="3"/>
+    <workbookView xWindow="32130" yWindow="2310" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PORTFOLIO" sheetId="1" r:id="rId1"/>
@@ -30,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="36">
   <si>
     <t>SEC_ID</t>
   </si>
@@ -125,9 +131,6 @@
     <t>WEIGHT</t>
   </si>
   <si>
-    <t>IND_CD</t>
-  </si>
-  <si>
     <t>ALL</t>
   </si>
   <si>
@@ -135,19 +138,19 @@
   </si>
   <si>
     <t>AVG_MAX_DRAWDOWN</t>
+  </si>
+  <si>
+    <t>VNQ+GSG+DBC</t>
+  </si>
+  <si>
+    <t>AGG+BND+JNK+TIP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="22">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -167,154 +170,9 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
-      <charset val="0"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -329,192 +187,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="4" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -537,251 +215,9 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -805,61 +241,17 @@
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1117,20 +509,20 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.57142857142857" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5714285714286" style="1" customWidth="1"/>
-    <col min="3" max="3" width="19.4285714285714" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.42857142857143" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.14285714285714" style="1"/>
+    <col min="1" max="1" width="9.5703125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.42578125" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1152,7 +544,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="3">
-        <v>0.035525</v>
+        <v>3.5525000000000001E-2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1163,7 +555,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="3">
-        <v>0.0336021842162834</v>
+        <v>3.3602184216283401E-2</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1174,7 +566,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="3">
-        <v>0.063561</v>
+        <v>6.3561000000000006E-2</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1185,7 +577,7 @@
         <v>6</v>
       </c>
       <c r="C5" s="3">
-        <v>0.07996</v>
+        <v>7.9960000000000003E-2</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1196,7 +588,7 @@
         <v>7</v>
       </c>
       <c r="C6" s="3">
-        <v>0.083065</v>
+        <v>8.3065E-2</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1218,7 +610,7 @@
         <v>9</v>
       </c>
       <c r="C8" s="3">
-        <v>0.043379</v>
+        <v>4.3379000000000001E-2</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1229,7 +621,7 @@
         <v>10</v>
       </c>
       <c r="C9" s="3">
-        <v>0.134797507460777</v>
+        <v>0.13479750746077701</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1262,7 +654,7 @@
         <v>13</v>
       </c>
       <c r="C12" s="3">
-        <v>0.165592522790983</v>
+        <v>0.16559252279098299</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1273,25 +665,23 @@
         <v>14</v>
       </c>
       <c r="C13" s="3">
-        <v>0.128723801461899</v>
+        <v>0.12872380146189899</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="6" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="26.2857142857143" style="1" customWidth="1"/>
-    <col min="2" max="2" width="20.2857142857143" style="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7142857142857" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.14285714285714" style="1"/>
+    <col min="1" max="1" width="26.28515625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1367,21 +757,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="6" outlineLevelCol="4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.1428571428571" style="4" customWidth="1"/>
-    <col min="2" max="2" width="24.7142857142857" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.1428571428571" style="1" customWidth="1"/>
-    <col min="4" max="5" width="8.42857142857143" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.14285714285714" style="1"/>
+    <col min="1" max="1" width="23.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" style="1" customWidth="1"/>
+    <col min="4" max="5" width="8.42578125" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -1413,83 +801,82 @@
         <v>0</v>
       </c>
       <c r="E2" s="7">
-        <v>1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="6" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7">
         <v>0</v>
       </c>
       <c r="E3" s="7">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7">
         <v>0</v>
       </c>
       <c r="E4" s="7">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" s="7">
-        <v>20</v>
-      </c>
+      <c r="C5" s="7"/>
       <c r="D5" s="7">
         <v>0</v>
       </c>
       <c r="E5" s="7">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="7">
+        <v>20</v>
+      </c>
+      <c r="D6" s="7">
+        <v>0</v>
+      </c>
+      <c r="E6" s="7">
         <v>0.09</v>
       </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="6"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="6"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:M13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="16384" width="9.14285714285714" style="1"/>
+    <col min="1" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -1538,40 +925,40 @@
         <v>3</v>
       </c>
       <c r="B2" s="3">
-        <v>0.002645</v>
+        <v>2.6450000000000002E-3</v>
       </c>
       <c r="C2" s="3">
-        <v>0.002579</v>
+        <v>2.5790000000000001E-3</v>
       </c>
       <c r="D2" s="3">
-        <v>-0.00074</v>
+        <v>-7.3999999999999999E-4</v>
       </c>
       <c r="E2" s="3">
-        <v>-0.00103</v>
+        <v>-1.0300000000000001E-3</v>
       </c>
       <c r="F2" s="3">
-        <v>0.001388</v>
+        <v>1.3879999999999999E-3</v>
       </c>
       <c r="G2" s="3">
-        <v>0.001121</v>
+        <v>1.121E-3</v>
       </c>
       <c r="H2" s="3">
-        <v>0.001928</v>
+        <v>1.928E-3</v>
       </c>
       <c r="I2" s="3">
-        <v>0.002027</v>
+        <v>2.0270000000000002E-3</v>
       </c>
       <c r="J2" s="3">
-        <v>0.004428</v>
+        <v>4.4279999999999996E-3</v>
       </c>
       <c r="K2" s="3">
-        <v>0.001236</v>
+        <v>1.2359999999999999E-3</v>
       </c>
       <c r="L2" s="3">
-        <v>0.001237</v>
+        <v>1.237E-3</v>
       </c>
       <c r="M2" s="3">
-        <v>0.001698</v>
+        <v>1.6980000000000001E-3</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1579,40 +966,40 @@
         <v>4</v>
       </c>
       <c r="B3" s="3">
-        <v>0.002579</v>
+        <v>2.5790000000000001E-3</v>
       </c>
       <c r="C3" s="3">
-        <v>0.002544</v>
+        <v>2.5439999999999998E-3</v>
       </c>
       <c r="D3" s="3">
-        <v>-0.0007</v>
+        <v>-6.9999999999999999E-4</v>
       </c>
       <c r="E3" s="3">
-        <v>-0.00098</v>
+        <v>-9.7999999999999997E-4</v>
       </c>
       <c r="F3" s="3">
-        <v>0.001368</v>
+        <v>1.3680000000000001E-3</v>
       </c>
       <c r="G3" s="3">
-        <v>0.001105</v>
+        <v>1.1050000000000001E-3</v>
       </c>
       <c r="H3" s="3">
-        <v>0.001898</v>
+        <v>1.8979999999999999E-3</v>
       </c>
       <c r="I3" s="3">
-        <v>0.001987</v>
+        <v>1.9870000000000001E-3</v>
       </c>
       <c r="J3" s="3">
-        <v>0.004355</v>
+        <v>4.3550000000000004E-3</v>
       </c>
       <c r="K3" s="3">
-        <v>0.001216</v>
+        <v>1.2160000000000001E-3</v>
       </c>
       <c r="L3" s="3">
-        <v>0.001214</v>
+        <v>1.214E-3</v>
       </c>
       <c r="M3" s="3">
-        <v>0.00166</v>
+        <v>1.66E-3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1620,40 +1007,40 @@
         <v>5</v>
       </c>
       <c r="B4" s="3">
-        <v>-0.00074</v>
+        <v>-7.3999999999999999E-4</v>
       </c>
       <c r="C4" s="3">
-        <v>-0.0007</v>
+        <v>-6.9999999999999999E-4</v>
       </c>
       <c r="D4" s="3">
-        <v>0.019542</v>
+        <v>1.9542E-2</v>
       </c>
       <c r="E4" s="3">
-        <v>0.0205683360963573</v>
+        <v>2.05683360963573E-2</v>
       </c>
       <c r="F4" s="3">
-        <v>0.000261</v>
+        <v>2.61E-4</v>
       </c>
       <c r="G4" s="3">
-        <v>0.002287</v>
+        <v>2.287E-3</v>
       </c>
       <c r="H4" s="3">
-        <v>0.000229</v>
+        <v>2.2900000000000001E-4</v>
       </c>
       <c r="I4" s="3">
-        <v>0.001463</v>
+        <v>1.4630000000000001E-3</v>
       </c>
       <c r="J4" s="3">
-        <v>-0.00155</v>
+        <v>-1.5499999999999999E-3</v>
       </c>
       <c r="K4" s="3">
-        <v>0.002231</v>
+        <v>2.2309999999999999E-3</v>
       </c>
       <c r="L4" s="3">
-        <v>0.000763</v>
+        <v>7.6300000000000001E-4</v>
       </c>
       <c r="M4" s="3">
-        <v>0.007383</v>
+        <v>7.3829999999999998E-3</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1661,40 +1048,40 @@
         <v>6</v>
       </c>
       <c r="B5" s="3">
-        <v>-0.00103</v>
+        <v>-1.0300000000000001E-3</v>
       </c>
       <c r="C5" s="3">
-        <v>-0.00098</v>
+        <v>-9.7999999999999997E-4</v>
       </c>
       <c r="D5" s="3">
-        <v>0.0205683360963573</v>
+        <v>2.05683360963573E-2</v>
       </c>
       <c r="E5" s="3">
-        <v>0.0232472402361165</v>
+        <v>2.32472402361165E-2</v>
       </c>
       <c r="F5" s="3">
-        <v>0.000187</v>
+        <v>1.8699999999999999E-4</v>
       </c>
       <c r="G5" s="3">
-        <v>0.001992</v>
+        <v>1.9919999999999998E-3</v>
       </c>
       <c r="H5" s="3">
-        <v>3.66764824017778e-5</v>
+        <v>3.6676482401777798E-5</v>
       </c>
       <c r="I5" s="3">
-        <v>0.001212</v>
+        <v>1.212E-3</v>
       </c>
       <c r="J5" s="3">
-        <v>-0.00237</v>
+        <v>-2.3700000000000001E-3</v>
       </c>
       <c r="K5" s="3">
-        <v>0.001931</v>
+        <v>1.931E-3</v>
       </c>
       <c r="L5" s="3">
-        <v>0.000742</v>
+        <v>7.4200000000000004E-4</v>
       </c>
       <c r="M5" s="3">
-        <v>0.00688</v>
+        <v>6.8799999999999998E-3</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1702,40 +1089,40 @@
         <v>7</v>
       </c>
       <c r="B6" s="3">
-        <v>0.001388</v>
+        <v>1.3879999999999999E-3</v>
       </c>
       <c r="C6" s="3">
-        <v>0.001368</v>
+        <v>1.3680000000000001E-3</v>
       </c>
       <c r="D6" s="3">
-        <v>0.000261</v>
+        <v>2.61E-4</v>
       </c>
       <c r="E6" s="3">
-        <v>0.000187</v>
+        <v>1.8699999999999999E-4</v>
       </c>
       <c r="F6" s="3">
-        <v>0.001761</v>
+        <v>1.761E-3</v>
       </c>
       <c r="G6" s="3">
-        <v>0.003496</v>
+        <v>3.496E-3</v>
       </c>
       <c r="H6" s="3">
-        <v>0.001084</v>
+        <v>1.0839999999999999E-3</v>
       </c>
       <c r="I6" s="3">
-        <v>0.004642</v>
+        <v>4.6420000000000003E-3</v>
       </c>
       <c r="J6" s="3">
-        <v>0.004281</v>
+        <v>4.2810000000000001E-3</v>
       </c>
       <c r="K6" s="3">
-        <v>0.003712</v>
+        <v>3.712E-3</v>
       </c>
       <c r="L6" s="3">
-        <v>0.002902</v>
+        <v>2.9020000000000001E-3</v>
       </c>
       <c r="M6" s="3">
-        <v>0.003031</v>
+        <v>3.0309999999999998E-3</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1743,40 +1130,40 @@
         <v>8</v>
       </c>
       <c r="B7" s="3">
-        <v>0.001121</v>
+        <v>1.121E-3</v>
       </c>
       <c r="C7" s="3">
-        <v>0.001105</v>
+        <v>1.1050000000000001E-3</v>
       </c>
       <c r="D7" s="3">
-        <v>0.002287</v>
+        <v>2.287E-3</v>
       </c>
       <c r="E7" s="3">
-        <v>0.001992</v>
+        <v>1.9919999999999998E-3</v>
       </c>
       <c r="F7" s="3">
-        <v>0.003496</v>
+        <v>3.496E-3</v>
       </c>
       <c r="G7" s="3">
-        <v>0.0159329139020716</v>
+        <v>1.5932913902071601E-2</v>
       </c>
       <c r="H7" s="3">
-        <v>0.00112</v>
+        <v>1.1199999999999999E-3</v>
       </c>
       <c r="I7" s="3">
-        <v>0.0146370778935135</v>
+        <v>1.4637077893513499E-2</v>
       </c>
       <c r="J7" s="3">
-        <v>0.008764</v>
+        <v>8.7639999999999992E-3</v>
       </c>
       <c r="K7" s="3">
-        <v>0.0162123249622911</v>
+        <v>1.6212324962291101E-2</v>
       </c>
       <c r="L7" s="3">
-        <v>0.0100167322798833</v>
+        <v>1.0016732279883299E-2</v>
       </c>
       <c r="M7" s="3">
-        <v>0.0103283881110823</v>
+        <v>1.03283881110823E-2</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1784,40 +1171,40 @@
         <v>9</v>
       </c>
       <c r="B8" s="3">
-        <v>0.001928</v>
+        <v>1.928E-3</v>
       </c>
       <c r="C8" s="3">
-        <v>0.001898</v>
+        <v>1.8979999999999999E-3</v>
       </c>
       <c r="D8" s="3">
-        <v>0.000229</v>
+        <v>2.2900000000000001E-4</v>
       </c>
       <c r="E8" s="3">
-        <v>3.66764824017778e-5</v>
+        <v>3.6676482401777798E-5</v>
       </c>
       <c r="F8" s="3">
-        <v>0.001084</v>
+        <v>1.0839999999999999E-3</v>
       </c>
       <c r="G8" s="3">
-        <v>0.00112</v>
+        <v>1.1199999999999999E-3</v>
       </c>
       <c r="H8" s="3">
-        <v>0.001741</v>
+        <v>1.7409999999999999E-3</v>
       </c>
       <c r="I8" s="3">
-        <v>0.001982</v>
+        <v>1.9819999999999998E-3</v>
       </c>
       <c r="J8" s="3">
-        <v>0.003293</v>
+        <v>3.2929999999999999E-3</v>
       </c>
       <c r="K8" s="3">
-        <v>0.001229</v>
+        <v>1.2290000000000001E-3</v>
       </c>
       <c r="L8" s="3">
-        <v>0.001231</v>
+        <v>1.2310000000000001E-3</v>
       </c>
       <c r="M8" s="3">
-        <v>0.001333</v>
+        <v>1.333E-3</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1825,40 +1212,40 @@
         <v>10</v>
       </c>
       <c r="B9" s="3">
-        <v>0.002027</v>
+        <v>2.0270000000000002E-3</v>
       </c>
       <c r="C9" s="3">
-        <v>0.001987</v>
+        <v>1.9870000000000001E-3</v>
       </c>
       <c r="D9" s="3">
-        <v>0.001463</v>
+        <v>1.4630000000000001E-3</v>
       </c>
       <c r="E9" s="3">
-        <v>0.001212</v>
+        <v>1.212E-3</v>
       </c>
       <c r="F9" s="3">
-        <v>0.004642</v>
+        <v>4.6420000000000003E-3</v>
       </c>
       <c r="G9" s="3">
-        <v>0.0146370778935135</v>
+        <v>1.4637077893513499E-2</v>
       </c>
       <c r="H9" s="3">
-        <v>0.001982</v>
+        <v>1.9819999999999998E-3</v>
       </c>
       <c r="I9" s="3">
-        <v>0.0250994148014261</v>
+        <v>2.50994148014261E-2</v>
       </c>
       <c r="J9" s="3">
-        <v>0.015679</v>
+        <v>1.5678999999999998E-2</v>
       </c>
       <c r="K9" s="3">
-        <v>0.0160505256438993</v>
+        <v>1.6050525643899301E-2</v>
       </c>
       <c r="L9" s="3">
-        <v>0.0149375934003046</v>
+        <v>1.4937593400304599E-2</v>
       </c>
       <c r="M9" s="3">
-        <v>0.0113351239056586</v>
+        <v>1.1335123905658599E-2</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1866,40 +1253,40 @@
         <v>11</v>
       </c>
       <c r="B10" s="3">
-        <v>0.004428</v>
+        <v>4.4279999999999996E-3</v>
       </c>
       <c r="C10" s="3">
-        <v>0.004355</v>
+        <v>4.3550000000000004E-3</v>
       </c>
       <c r="D10" s="3">
-        <v>-0.00155</v>
+        <v>-1.5499999999999999E-3</v>
       </c>
       <c r="E10" s="3">
-        <v>-0.00237</v>
+        <v>-2.3700000000000001E-3</v>
       </c>
       <c r="F10" s="3">
-        <v>0.004281</v>
+        <v>4.2810000000000001E-3</v>
       </c>
       <c r="G10" s="3">
-        <v>0.008764</v>
+        <v>8.7639999999999992E-3</v>
       </c>
       <c r="H10" s="3">
-        <v>0.003293</v>
+        <v>3.2929999999999999E-3</v>
       </c>
       <c r="I10" s="3">
-        <v>0.015679</v>
+        <v>1.5678999999999998E-2</v>
       </c>
       <c r="J10" s="3">
-        <v>0.025143</v>
+        <v>2.5142999999999999E-2</v>
       </c>
       <c r="K10" s="3">
-        <v>0.009549</v>
+        <v>9.5490000000000002E-3</v>
       </c>
       <c r="L10" s="3">
-        <v>0.0112482475531891</v>
+        <v>1.12482475531891E-2</v>
       </c>
       <c r="M10" s="3">
-        <v>0.007726</v>
+        <v>7.7260000000000002E-3</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1907,40 +1294,40 @@
         <v>12</v>
       </c>
       <c r="B11" s="3">
-        <v>0.001236</v>
+        <v>1.2359999999999999E-3</v>
       </c>
       <c r="C11" s="3">
-        <v>0.001216</v>
+        <v>1.2160000000000001E-3</v>
       </c>
       <c r="D11" s="3">
-        <v>0.002231</v>
+        <v>2.2309999999999999E-3</v>
       </c>
       <c r="E11" s="3">
-        <v>0.001931</v>
+        <v>1.931E-3</v>
       </c>
       <c r="F11" s="3">
-        <v>0.003712</v>
+        <v>3.712E-3</v>
       </c>
       <c r="G11" s="3">
-        <v>0.0162123249622911</v>
+        <v>1.6212324962291101E-2</v>
       </c>
       <c r="H11" s="3">
-        <v>0.001229</v>
+        <v>1.2290000000000001E-3</v>
       </c>
       <c r="I11" s="3">
-        <v>0.0160505256438993</v>
+        <v>1.6050525643899301E-2</v>
       </c>
       <c r="J11" s="3">
-        <v>0.009549</v>
+        <v>9.5490000000000002E-3</v>
       </c>
       <c r="K11" s="3">
-        <v>0.0166709814564034</v>
+        <v>1.6670981456403399E-2</v>
       </c>
       <c r="L11" s="3">
-        <v>0.0106700001366691</v>
+        <v>1.06700001366691E-2</v>
       </c>
       <c r="M11" s="3">
-        <v>0.010688</v>
+        <v>1.0688E-2</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -1948,40 +1335,40 @@
         <v>13</v>
       </c>
       <c r="B12" s="3">
-        <v>0.001237</v>
+        <v>1.237E-3</v>
       </c>
       <c r="C12" s="3">
-        <v>0.001214</v>
+        <v>1.214E-3</v>
       </c>
       <c r="D12" s="3">
-        <v>0.000763</v>
+        <v>7.6300000000000001E-4</v>
       </c>
       <c r="E12" s="3">
-        <v>0.000742</v>
+        <v>7.4200000000000004E-4</v>
       </c>
       <c r="F12" s="3">
-        <v>0.002902</v>
+        <v>2.9020000000000001E-3</v>
       </c>
       <c r="G12" s="3">
-        <v>0.0100167322798833</v>
+        <v>1.0016732279883299E-2</v>
       </c>
       <c r="H12" s="3">
-        <v>0.001231</v>
+        <v>1.2310000000000001E-3</v>
       </c>
       <c r="I12" s="3">
-        <v>0.0149375934003046</v>
+        <v>1.4937593400304599E-2</v>
       </c>
       <c r="J12" s="3">
-        <v>0.0112482475531891</v>
+        <v>1.12482475531891E-2</v>
       </c>
       <c r="K12" s="3">
-        <v>0.0106700001366691</v>
+        <v>1.06700001366691E-2</v>
       </c>
       <c r="L12" s="3">
-        <v>0.0111635614859139</v>
+        <v>1.11635614859139E-2</v>
       </c>
       <c r="M12" s="3">
-        <v>0.007143</v>
+        <v>7.143E-3</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -1989,44 +1376,43 @@
         <v>14</v>
       </c>
       <c r="B13" s="3">
-        <v>0.001698</v>
+        <v>1.6980000000000001E-3</v>
       </c>
       <c r="C13" s="3">
-        <v>0.00166</v>
+        <v>1.66E-3</v>
       </c>
       <c r="D13" s="3">
-        <v>0.007383</v>
+        <v>7.3829999999999998E-3</v>
       </c>
       <c r="E13" s="3">
-        <v>0.00688</v>
+        <v>6.8799999999999998E-3</v>
       </c>
       <c r="F13" s="3">
-        <v>0.003031</v>
+        <v>3.0309999999999998E-3</v>
       </c>
       <c r="G13" s="3">
-        <v>0.0103283881110823</v>
+        <v>1.03283881110823E-2</v>
       </c>
       <c r="H13" s="3">
-        <v>0.001333</v>
+        <v>1.333E-3</v>
       </c>
       <c r="I13" s="3">
-        <v>0.0113351239056586</v>
+        <v>1.1335123905658599E-2</v>
       </c>
       <c r="J13" s="3">
-        <v>0.007726</v>
+        <v>7.7260000000000002E-3</v>
       </c>
       <c r="K13" s="3">
-        <v>0.010688</v>
+        <v>1.0688E-2</v>
       </c>
       <c r="L13" s="3">
-        <v>0.007143</v>
+        <v>7.143E-3</v>
       </c>
       <c r="M13" s="3">
-        <v>0.021645</v>
+        <v>2.1645000000000001E-2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
enriched covar matrix output; added GLD to portfolio.
</commit_message>
<xml_diff>
--- a/template_etf_input.xlsx
+++ b/template_etf_input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zypub\PycharmProjects\sport\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C910532F-100F-4B6D-A660-F1A1346C346F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{407473D9-566C-41A6-A6BE-6DB6B618020A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32130" yWindow="2310" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PORTFOLIO" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="60">
   <si>
     <t>SEC_ID</t>
   </si>
@@ -140,10 +140,82 @@
     <t>AVG_MAX_DRAWDOWN</t>
   </si>
   <si>
-    <t>VNQ+GSG+DBC</t>
-  </si>
-  <si>
     <t>AGG+BND+JNK+TIP</t>
+  </si>
+  <si>
+    <t>VNQ+GSG+DBC+GLD</t>
+  </si>
+  <si>
+    <t>GLD</t>
+  </si>
+  <si>
+    <t>0.032537431288129526</t>
+  </si>
+  <si>
+    <t>0.011459520589468452</t>
+  </si>
+  <si>
+    <t>0.011595373671026208</t>
+  </si>
+  <si>
+    <t>0.012569611975650279</t>
+  </si>
+  <si>
+    <t>0.023085843738953664</t>
+  </si>
+  <si>
+    <t>0.010180645469752685</t>
+  </si>
+  <si>
+    <t>0.013268225126761934</t>
+  </si>
+  <si>
+    <t>0.015008075295334872</t>
+  </si>
+  <si>
+    <t>0.013409821190671148</t>
+  </si>
+  <si>
+    <t>0.011624646169794636</t>
+  </si>
+  <si>
+    <t>0.013529248999326018</t>
+  </si>
+  <si>
+    <t>0.010864154513541007</t>
+  </si>
+  <si>
+    <t>0.011937284061472035</t>
+  </si>
+  <si>
+    <t>0.010851445648324149</t>
+  </si>
+  <si>
+    <t>0.011127113165479229</t>
+  </si>
+  <si>
+    <t>0.036240350534241565</t>
+  </si>
+  <si>
+    <t>0.026072029771675862</t>
+  </si>
+  <si>
+    <t>0.023436566516623594</t>
+  </si>
+  <si>
+    <t>0.035820487687706966</t>
+  </si>
+  <si>
+    <t>0.024305537173579216</t>
+  </si>
+  <si>
+    <t>0.026941790609259803</t>
+  </si>
+  <si>
+    <t>0.024243960727657807</t>
+  </si>
+  <si>
+    <t>0.017660005856369704</t>
   </si>
 </sst>
 </file>
@@ -515,7 +587,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.5703125" style="1" customWidth="1"/>
@@ -666,6 +738,17 @@
       </c>
       <c r="C13" s="3">
         <v>0.12872380146189899</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>
@@ -806,7 +889,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>30</v>
@@ -821,7 +904,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>30</v>
@@ -873,13 +956,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -893,523 +976,606 @@
         <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:14">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="3">
-        <v>2.6450000000000002E-3</v>
+        <v>3.7115291583607502E-3</v>
       </c>
       <c r="C2" s="3">
-        <v>2.5790000000000001E-3</v>
+        <v>3.6408335394247301E-3</v>
       </c>
       <c r="D2" s="3">
-        <v>-7.3999999999999999E-4</v>
+        <v>-7.2498130773206401E-5</v>
       </c>
       <c r="E2" s="3">
-        <v>-1.0300000000000001E-3</v>
+        <v>2.7125910528314101E-3</v>
       </c>
       <c r="F2" s="3">
-        <v>1.3879999999999999E-3</v>
+        <v>-3.6614282733737701E-4</v>
       </c>
       <c r="G2" s="3">
-        <v>1.121E-3</v>
+        <v>2.3400994051311899E-3</v>
       </c>
       <c r="H2" s="3">
-        <v>1.928E-3</v>
+        <v>1.83130829830582E-3</v>
       </c>
       <c r="I2" s="3">
-        <v>2.0270000000000002E-3</v>
+        <v>3.0390220068359001E-3</v>
       </c>
       <c r="J2" s="3">
-        <v>4.4279999999999996E-3</v>
+        <v>2.4203837167996799E-3</v>
       </c>
       <c r="K2" s="3">
-        <v>1.2359999999999999E-3</v>
+        <v>4.8319996481848001E-3</v>
       </c>
       <c r="L2" s="3">
-        <v>1.237E-3</v>
+        <v>1.93920815897569E-3</v>
       </c>
       <c r="M2" s="3">
-        <v>1.6980000000000001E-3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
+        <v>1.5452661053251E-3</v>
+      </c>
+      <c r="N2" s="3">
+        <v>2.0909944007674302E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="3">
-        <v>2.5790000000000001E-3</v>
+        <v>3.6408335394247301E-3</v>
       </c>
       <c r="C3" s="3">
-        <v>2.5439999999999998E-3</v>
+        <v>3.6437570574715801E-3</v>
       </c>
       <c r="D3" s="3">
-        <v>-6.9999999999999999E-4</v>
+        <v>-1.57056354578347E-4</v>
       </c>
       <c r="E3" s="3">
-        <v>-9.7999999999999997E-4</v>
+        <v>2.6630410315600199E-3</v>
       </c>
       <c r="F3" s="3">
-        <v>1.3680000000000001E-3</v>
+        <v>-4.6257325195476801E-4</v>
       </c>
       <c r="G3" s="3">
-        <v>1.1050000000000001E-3</v>
+        <v>2.3096642092918498E-3</v>
       </c>
       <c r="H3" s="3">
-        <v>1.8979999999999999E-3</v>
+        <v>1.77638699956494E-3</v>
       </c>
       <c r="I3" s="3">
-        <v>1.9870000000000001E-3</v>
+        <v>2.99570836199487E-3</v>
       </c>
       <c r="J3" s="3">
-        <v>4.3550000000000004E-3</v>
+        <v>2.2803186399938898E-3</v>
       </c>
       <c r="K3" s="3">
-        <v>1.2160000000000001E-3</v>
+        <v>4.7696243380145296E-3</v>
       </c>
       <c r="L3" s="3">
-        <v>1.214E-3</v>
+        <v>1.87362161960668E-3</v>
       </c>
       <c r="M3" s="3">
-        <v>1.66E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
+        <v>1.5181022398620999E-3</v>
+      </c>
+      <c r="N3" s="3">
+        <v>1.9997517938450502E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="3">
-        <v>-7.3999999999999999E-4</v>
+        <v>-7.2498130773206401E-5</v>
       </c>
       <c r="C4" s="3">
-        <v>-6.9999999999999999E-4</v>
+        <v>-1.57056354578347E-4</v>
       </c>
       <c r="D4" s="3">
-        <v>1.9542E-2</v>
+        <v>2.8683766645616299E-2</v>
       </c>
       <c r="E4" s="3">
-        <v>2.05683360963573E-2</v>
-      </c>
-      <c r="F4" s="3">
-        <v>2.61E-4</v>
+        <v>9.9882826454315201E-3</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>37</v>
       </c>
       <c r="G4" s="3">
-        <v>2.287E-3</v>
-      </c>
-      <c r="H4" s="3">
-        <v>2.2900000000000001E-4</v>
+        <v>3.85875717752992E-3</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>38</v>
       </c>
       <c r="I4" s="3">
-        <v>1.4630000000000001E-3</v>
+        <v>1.4289293243873501E-3</v>
       </c>
       <c r="J4" s="3">
-        <v>-1.5499999999999999E-3</v>
+        <v>1.2980949953789799E-2</v>
       </c>
       <c r="K4" s="3">
-        <v>2.2309999999999999E-3</v>
-      </c>
-      <c r="L4" s="3">
-        <v>7.6300000000000001E-4</v>
+        <v>7.8705787811896404E-3</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>39</v>
       </c>
       <c r="M4" s="3">
-        <v>7.3829999999999998E-3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
+        <v>9.8858957022140894E-3</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="3">
+        <v>2.7125910528314101E-3</v>
+      </c>
+      <c r="C5" s="3">
+        <v>2.6630410315600199E-3</v>
+      </c>
+      <c r="D5" s="3">
+        <v>9.9882826454315201E-3</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F5" s="3">
+        <v>9.8658583101165001E-3</v>
+      </c>
+      <c r="G5" s="3">
+        <v>2.9412274163600699E-3</v>
+      </c>
+      <c r="H5" s="3">
+        <v>5.4454844750175101E-3</v>
+      </c>
+      <c r="I5" s="3">
+        <v>2.9249609978923299E-3</v>
+      </c>
+      <c r="J5" s="3">
+        <v>5.0593295135019601E-3</v>
+      </c>
+      <c r="K5" s="3">
+        <v>6.9018945197713098E-3</v>
+      </c>
+      <c r="L5" s="3">
+        <v>5.5665203410786004E-3</v>
+      </c>
+      <c r="M5" s="3">
+        <v>4.2430786443573704E-3</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="3">
-        <v>-1.0300000000000001E-3</v>
-      </c>
-      <c r="C5" s="3">
-        <v>-9.7999999999999997E-4</v>
-      </c>
-      <c r="D5" s="3">
-        <v>2.05683360963573E-2</v>
-      </c>
-      <c r="E5" s="3">
-        <v>2.32472402361165E-2</v>
-      </c>
-      <c r="F5" s="3">
-        <v>1.8699999999999999E-4</v>
-      </c>
-      <c r="G5" s="3">
-        <v>1.9919999999999998E-3</v>
-      </c>
-      <c r="H5" s="3">
-        <v>3.6676482401777798E-5</v>
-      </c>
-      <c r="I5" s="3">
-        <v>1.212E-3</v>
-      </c>
-      <c r="J5" s="3">
-        <v>-2.3700000000000001E-3</v>
-      </c>
-      <c r="K5" s="3">
-        <v>1.931E-3</v>
-      </c>
-      <c r="L5" s="3">
-        <v>7.4200000000000004E-4</v>
-      </c>
-      <c r="M5" s="3">
-        <v>6.8799999999999998E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="3" t="s">
+      <c r="B6" s="3">
+        <v>-3.6614282733737701E-4</v>
+      </c>
+      <c r="C6" s="3">
+        <v>-4.6257325195476801E-4</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" s="3">
+        <v>9.8658583101165001E-3</v>
+      </c>
+      <c r="F6" s="3">
+        <v>3.92340474963144E-2</v>
+      </c>
+      <c r="G6" s="3">
+        <v>4.3356850507041004E-3</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" s="3">
+        <v>1.4730017833216901E-3</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K6" s="3">
+        <v>8.6976746827577296E-3</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="3">
-        <v>1.3879999999999999E-3</v>
-      </c>
-      <c r="C6" s="3">
-        <v>1.3680000000000001E-3</v>
-      </c>
-      <c r="D6" s="3">
-        <v>2.61E-4</v>
-      </c>
-      <c r="E6" s="3">
-        <v>1.8699999999999999E-4</v>
-      </c>
-      <c r="F6" s="3">
-        <v>1.761E-3</v>
-      </c>
-      <c r="G6" s="3">
-        <v>3.496E-3</v>
-      </c>
-      <c r="H6" s="3">
-        <v>1.0839999999999999E-3</v>
-      </c>
-      <c r="I6" s="3">
-        <v>4.6420000000000003E-3</v>
-      </c>
-      <c r="J6" s="3">
-        <v>4.2810000000000001E-3</v>
-      </c>
-      <c r="K6" s="3">
-        <v>3.712E-3</v>
-      </c>
-      <c r="L6" s="3">
-        <v>2.9020000000000001E-3</v>
-      </c>
-      <c r="M6" s="3">
-        <v>3.0309999999999998E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="3" t="s">
+      <c r="B7" s="3">
+        <v>2.3400994051311899E-3</v>
+      </c>
+      <c r="C7" s="3">
+        <v>2.3096642092918498E-3</v>
+      </c>
+      <c r="D7" s="3">
+        <v>3.85875717752992E-3</v>
+      </c>
+      <c r="E7" s="3">
+        <v>2.9412274163600699E-3</v>
+      </c>
+      <c r="F7" s="3">
+        <v>4.3356850507041004E-3</v>
+      </c>
+      <c r="G7" s="3">
+        <v>5.56408546857033E-3</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" s="3">
+        <v>2.0177017423778699E-3</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="M7" s="3">
+        <v>8.48210923777124E-3</v>
+      </c>
+      <c r="N7" s="3">
+        <v>8.23137089257725E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="3">
-        <v>1.121E-3</v>
-      </c>
-      <c r="C7" s="3">
-        <v>1.1050000000000001E-3</v>
-      </c>
-      <c r="D7" s="3">
-        <v>2.287E-3</v>
-      </c>
-      <c r="E7" s="3">
-        <v>1.9919999999999998E-3</v>
-      </c>
-      <c r="F7" s="3">
-        <v>3.496E-3</v>
-      </c>
-      <c r="G7" s="3">
-        <v>1.5932913902071601E-2</v>
-      </c>
-      <c r="H7" s="3">
-        <v>1.1199999999999999E-3</v>
-      </c>
-      <c r="I7" s="3">
-        <v>1.4637077893513499E-2</v>
-      </c>
-      <c r="J7" s="3">
-        <v>8.7639999999999992E-3</v>
-      </c>
-      <c r="K7" s="3">
-        <v>1.6212324962291101E-2</v>
-      </c>
-      <c r="L7" s="3">
-        <v>1.0016732279883299E-2</v>
-      </c>
-      <c r="M7" s="3">
-        <v>1.03283881110823E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="3" t="s">
+      <c r="B8" s="3">
+        <v>1.83130829830582E-3</v>
+      </c>
+      <c r="C8" s="3">
+        <v>1.77638699956494E-3</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="3">
+        <v>5.4454844750175101E-3</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H8" s="3">
+        <v>3.6045724137222297E-2</v>
+      </c>
+      <c r="I8" s="3">
+        <v>1.88072853294257E-3</v>
+      </c>
+      <c r="J8" s="3">
+        <v>3.4431549859675899E-2</v>
+      </c>
+      <c r="K8" s="3">
+        <v>2.6059888470578999E-2</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="N8" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="3">
-        <v>1.928E-3</v>
-      </c>
-      <c r="C8" s="3">
-        <v>1.8979999999999999E-3</v>
-      </c>
-      <c r="D8" s="3">
-        <v>2.2900000000000001E-4</v>
-      </c>
-      <c r="E8" s="3">
-        <v>3.6676482401777798E-5</v>
-      </c>
-      <c r="F8" s="3">
-        <v>1.0839999999999999E-3</v>
-      </c>
-      <c r="G8" s="3">
-        <v>1.1199999999999999E-3</v>
-      </c>
-      <c r="H8" s="3">
-        <v>1.7409999999999999E-3</v>
-      </c>
-      <c r="I8" s="3">
-        <v>1.9819999999999998E-3</v>
-      </c>
-      <c r="J8" s="3">
-        <v>3.2929999999999999E-3</v>
-      </c>
-      <c r="K8" s="3">
-        <v>1.2290000000000001E-3</v>
-      </c>
-      <c r="L8" s="3">
-        <v>1.2310000000000001E-3</v>
-      </c>
-      <c r="M8" s="3">
-        <v>1.333E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="3" t="s">
+      <c r="B9" s="3">
+        <v>3.0390220068359001E-3</v>
+      </c>
+      <c r="C9" s="3">
+        <v>2.99570836199487E-3</v>
+      </c>
+      <c r="D9" s="3">
+        <v>1.4289293243873501E-3</v>
+      </c>
+      <c r="E9" s="3">
+        <v>2.9249609978923299E-3</v>
+      </c>
+      <c r="F9" s="3">
+        <v>1.4730017833216901E-3</v>
+      </c>
+      <c r="G9" s="3">
+        <v>2.0177017423778699E-3</v>
+      </c>
+      <c r="H9" s="3">
+        <v>1.88072853294257E-3</v>
+      </c>
+      <c r="I9" s="3">
+        <v>3.4351965552476401E-3</v>
+      </c>
+      <c r="J9" s="3">
+        <v>2.3501762321967799E-3</v>
+      </c>
+      <c r="K9" s="3">
+        <v>4.1469136397492296E-3</v>
+      </c>
+      <c r="L9" s="3">
+        <v>1.95099172743697E-3</v>
+      </c>
+      <c r="M9" s="3">
+        <v>1.6857658430670601E-3</v>
+      </c>
+      <c r="N9" s="3">
+        <v>1.76965310409983E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="3">
-        <v>2.0270000000000002E-3</v>
-      </c>
-      <c r="C9" s="3">
-        <v>1.9870000000000001E-3</v>
-      </c>
-      <c r="D9" s="3">
-        <v>1.4630000000000001E-3</v>
-      </c>
-      <c r="E9" s="3">
-        <v>1.212E-3</v>
-      </c>
-      <c r="F9" s="3">
-        <v>4.6420000000000003E-3</v>
-      </c>
-      <c r="G9" s="3">
-        <v>1.4637077893513499E-2</v>
-      </c>
-      <c r="H9" s="3">
-        <v>1.9819999999999998E-3</v>
-      </c>
-      <c r="I9" s="3">
-        <v>2.50994148014261E-2</v>
-      </c>
-      <c r="J9" s="3">
-        <v>1.5678999999999998E-2</v>
-      </c>
-      <c r="K9" s="3">
-        <v>1.6050525643899301E-2</v>
-      </c>
-      <c r="L9" s="3">
-        <v>1.4937593400304599E-2</v>
-      </c>
-      <c r="M9" s="3">
-        <v>1.1335123905658599E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="3" t="s">
+      <c r="B10" s="3">
+        <v>2.4203837167996799E-3</v>
+      </c>
+      <c r="C10" s="3">
+        <v>2.2803186399938898E-3</v>
+      </c>
+      <c r="D10" s="3">
+        <v>1.2980949953789799E-2</v>
+      </c>
+      <c r="E10" s="3">
+        <v>5.0593295135019601E-3</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="H10" s="3">
+        <v>3.4431549859675899E-2</v>
+      </c>
+      <c r="I10" s="3">
+        <v>2.3501762321967799E-3</v>
+      </c>
+      <c r="J10" s="3">
+        <v>4.52857284499825E-2</v>
+      </c>
+      <c r="K10" s="3">
+        <v>3.3096160519821498E-2</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="M10" s="3">
+        <v>3.00299777551142E-2</v>
+      </c>
+      <c r="N10" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="3">
-        <v>4.4279999999999996E-3</v>
-      </c>
-      <c r="C10" s="3">
-        <v>4.3550000000000004E-3</v>
-      </c>
-      <c r="D10" s="3">
-        <v>-1.5499999999999999E-3</v>
-      </c>
-      <c r="E10" s="3">
-        <v>-2.3700000000000001E-3</v>
-      </c>
-      <c r="F10" s="3">
-        <v>4.2810000000000001E-3</v>
-      </c>
-      <c r="G10" s="3">
-        <v>8.7639999999999992E-3</v>
-      </c>
-      <c r="H10" s="3">
-        <v>3.2929999999999999E-3</v>
-      </c>
-      <c r="I10" s="3">
-        <v>1.5678999999999998E-2</v>
-      </c>
-      <c r="J10" s="3">
-        <v>2.5142999999999999E-2</v>
-      </c>
-      <c r="K10" s="3">
-        <v>9.5490000000000002E-3</v>
-      </c>
-      <c r="L10" s="3">
-        <v>1.12482475531891E-2</v>
-      </c>
-      <c r="M10" s="3">
-        <v>7.7260000000000002E-3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
-      <c r="A11" s="3" t="s">
+      <c r="B11" s="3">
+        <v>4.8319996481848001E-3</v>
+      </c>
+      <c r="C11" s="3">
+        <v>4.7696243380145296E-3</v>
+      </c>
+      <c r="D11" s="3">
+        <v>7.8705787811896404E-3</v>
+      </c>
+      <c r="E11" s="3">
+        <v>6.9018945197713098E-3</v>
+      </c>
+      <c r="F11" s="3">
+        <v>8.6976746827577296E-3</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H11" s="3">
+        <v>2.6059888470578999E-2</v>
+      </c>
+      <c r="I11" s="3">
+        <v>4.1469136397492296E-3</v>
+      </c>
+      <c r="J11" s="3">
+        <v>3.3096160519821498E-2</v>
+      </c>
+      <c r="K11" s="3">
+        <v>4.01398854922577E-2</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="N11" s="3">
+        <v>1.9326548764291501E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="3">
-        <v>1.2359999999999999E-3</v>
-      </c>
-      <c r="C11" s="3">
-        <v>1.2160000000000001E-3</v>
-      </c>
-      <c r="D11" s="3">
-        <v>2.2309999999999999E-3</v>
-      </c>
-      <c r="E11" s="3">
-        <v>1.931E-3</v>
-      </c>
-      <c r="F11" s="3">
-        <v>3.712E-3</v>
-      </c>
-      <c r="G11" s="3">
-        <v>1.6212324962291101E-2</v>
-      </c>
-      <c r="H11" s="3">
-        <v>1.2290000000000001E-3</v>
-      </c>
-      <c r="I11" s="3">
-        <v>1.6050525643899301E-2</v>
-      </c>
-      <c r="J11" s="3">
-        <v>9.5490000000000002E-3</v>
-      </c>
-      <c r="K11" s="3">
-        <v>1.6670981456403399E-2</v>
-      </c>
-      <c r="L11" s="3">
-        <v>1.06700001366691E-2</v>
-      </c>
-      <c r="M11" s="3">
-        <v>1.0688E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13">
-      <c r="A12" s="3" t="s">
+      <c r="B12" s="3">
+        <v>1.93920815897569E-3</v>
+      </c>
+      <c r="C12" s="3">
+        <v>1.87362161960668E-3</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E12" s="3">
+        <v>5.5665203410786004E-3</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I12" s="3">
+        <v>1.95099172743697E-3</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="L12" s="3">
+        <v>3.6686326261697801E-2</v>
+      </c>
+      <c r="M12" s="3">
+        <v>2.6519856618326201E-2</v>
+      </c>
+      <c r="N12" s="3">
+        <v>2.3958202123732002E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="A13" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="3">
-        <v>1.237E-3</v>
-      </c>
-      <c r="C12" s="3">
-        <v>1.214E-3</v>
-      </c>
-      <c r="D12" s="3">
-        <v>7.6300000000000001E-4</v>
-      </c>
-      <c r="E12" s="3">
-        <v>7.4200000000000004E-4</v>
-      </c>
-      <c r="F12" s="3">
-        <v>2.9020000000000001E-3</v>
-      </c>
-      <c r="G12" s="3">
-        <v>1.0016732279883299E-2</v>
-      </c>
-      <c r="H12" s="3">
-        <v>1.2310000000000001E-3</v>
-      </c>
-      <c r="I12" s="3">
-        <v>1.4937593400304599E-2</v>
-      </c>
-      <c r="J12" s="3">
-        <v>1.12482475531891E-2</v>
-      </c>
-      <c r="K12" s="3">
-        <v>1.06700001366691E-2</v>
-      </c>
-      <c r="L12" s="3">
-        <v>1.11635614859139E-2</v>
-      </c>
-      <c r="M12" s="3">
-        <v>7.143E-3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13">
-      <c r="A13" s="3" t="s">
+      <c r="B13" s="3">
+        <v>1.5452661053251E-3</v>
+      </c>
+      <c r="C13" s="3">
+        <v>1.5181022398620999E-3</v>
+      </c>
+      <c r="D13" s="3">
+        <v>9.8858957022140894E-3</v>
+      </c>
+      <c r="E13" s="3">
+        <v>4.2430786443573704E-3</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G13" s="3">
+        <v>8.48210923777124E-3</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I13" s="3">
+        <v>1.6857658430670601E-3</v>
+      </c>
+      <c r="J13" s="3">
+        <v>3.00299777551142E-2</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="L13" s="3">
+        <v>2.6519856618326201E-2</v>
+      </c>
+      <c r="M13" s="3">
+        <v>2.3949976507979701E-2</v>
+      </c>
+      <c r="N13" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="3">
-        <v>1.6980000000000001E-3</v>
-      </c>
-      <c r="C13" s="3">
-        <v>1.66E-3</v>
-      </c>
-      <c r="D13" s="3">
-        <v>7.3829999999999998E-3</v>
-      </c>
-      <c r="E13" s="3">
-        <v>6.8799999999999998E-3</v>
-      </c>
-      <c r="F13" s="3">
-        <v>3.0309999999999998E-3</v>
-      </c>
-      <c r="G13" s="3">
-        <v>1.03283881110823E-2</v>
-      </c>
-      <c r="H13" s="3">
-        <v>1.333E-3</v>
-      </c>
-      <c r="I13" s="3">
-        <v>1.1335123905658599E-2</v>
-      </c>
-      <c r="J13" s="3">
-        <v>7.7260000000000002E-3</v>
-      </c>
-      <c r="K13" s="3">
-        <v>1.0688E-2</v>
-      </c>
-      <c r="L13" s="3">
-        <v>7.143E-3</v>
-      </c>
-      <c r="M13" s="3">
-        <v>2.1645000000000001E-2</v>
+      <c r="B14" s="3">
+        <v>2.0909944007674302E-3</v>
+      </c>
+      <c r="C14" s="3">
+        <v>1.9997517938450502E-3</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="G14" s="3">
+        <v>8.23137089257725E-3</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="I14" s="3">
+        <v>1.76965310409983E-3</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="K14" s="3">
+        <v>1.9326548764291501E-2</v>
+      </c>
+      <c r="L14" s="3">
+        <v>2.3958202123732002E-2</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="N14" s="3">
+        <v>3.2557767546260899E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>